<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-06 Les chaussettes du radiateur
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-06.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-06.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut les chaussettes de laine près du radiateur. La tour de cubes tombe dessus. Elle cherche, met cubes et voiture dans la caisse. Les chaussettes apparaissent. Pieds au chaud, livre du canard.</t>
+          <t>Au campement du radiateur, un éclat de laine brille sur le métal. Mila veut les chaussettes chaudes, maintenant. La tour penche : les cubes tombent sur la laine. Elle cherche le canapé, les paumes, puis saisit toute la pile : les cubes s'éparpillent. Elle refuse de foncer, pose un cube, retrouve la laine. Sur l'orteil, l'éclat de laine tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur chante un tout petit air. Psss. Des chaussettes de laine attendent. Elles sont épaisses, près du canapé. Elles sentent le linge propre. Les chaussettes sont chaudes, papa. Oui, on les laisse près du chaud. Une caisse en bois est au salon. Elle sent un peu la forêt. En ce moment, Mila est près du canapé. Elle touche un cube. Le cube est lisse. Il est chaud, papa. C'est le radiateur, Mila. Je fais une petite tour. Une tour, avant les chaussettes ? Oui, une tour petite. Mila pose un cube. Puis un autre cube. Clic. Elle fait une petite tour. Ta tour est jolie. Elle est petite, papa. Mila pose un cube rouge. Clic. La tour grandit un peu. Ses pieds sont près du radiateur. Après, les chaussettes chaudes. Oui, pour les orteils. Mila pose encore un cube. La tour penche vers les chaussettes. Deux cubes glissent. Ils tombent sur la laine. Oh. La tour a bougé. Où sont mes chaussettes ? Sur le canapé, peut-être ? Mila monte un genou. Le coussin est vide. Dans mes mains ? Elle ouvre les paumes. Rien. Elles sont perdues. Les cubes sont encore au pied. Je veux voir dessous. Mila prend un cube. Elle le pose dans la caisse. Toc. Une petite voiture attend aussi. Elle va dans la caisse. Toc.</t>
+          <t>Le métal du radiateur fait psss. Une lampe ronde pose un halo. Mila connaît ce salon, le soir. Un détail paraît nouveau, sur le métal. Au campement du radiateur, ça sent le bois. Des chaussettes de laine attendent. Elles sont épaisses, près du canapé. Sur le bord, un éclat de laine brille. Il est petit, papa. C'est un éclat de laine. La laine sent le linge propre. Les chaussettes sont chaudes, Mila. On les laisse près du chaud. Une caisse en bois est là. Elle sent un peu la forêt. Le tapis est froid, sous les orteils. J'ai froid aux pieds ! Je veux les chaussettes, maintenant ! Avant la tour de cubes ? Non, les chaussettes d'abord ! En ce moment, Mila saisit la laine. La laine est chaude, un peu lourde. Un cube rouge attend au sol. Une tour petite, aussi ! Elle pose un cube trop vite. Ça fait clic, contre le tapis. Puis un cube jaune. Ça fait clic, contre le rouge. Ta tour est jolie. Elle est petite, papa. Mila pose un cube de plus. La tour penche vers la laine. Deux cubes glissent. Ils tombent sur les chaussettes. Oh. Le sourire de Mila disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Où sont mes chaussettes ? Sur le canapé, peut-être ? Mila monte un genou. Le coussin est vide. Dans mes mains ? Elle ouvre les paumes. Rien. Elles sont perdues. Je prends tout, d'un coup ! Elle saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur chante un tout petit air. Psss. Des chaussettes de laine attendent. Elles sont épaisses, près du canapé. Elles sentent le linge propre. Les chaussettes sont chaudes, papa. Oui, on les laisse près du chaud. Une caisse en bois est au salon. Elle sent un peu la forêt. En ce moment, Mila est près du canapé. Elle touche un cube. Le cube est lisse. Il est chaud, papa. C'est le radiateur, Mila. Je fais une petite tour. Une tour, avant les chaussettes ? Oui, une tour petite. Mila pose un cube. Puis un autre cube. Clic. Elle fait une petite tour. Ta tour est jolie. Elle est petite, papa. Mila pose un cube rouge. Clic. La tour grandit un peu. Ses pieds sont près du radiateur. Après, les chaussettes chaudes. Oui, pour les orteils. Mila pose encore un cube. La tour penche vers les chaussettes. Deux cubes glissent. Ils tombent sur la laine. Oh. La tour a bougé. Où sont mes chaussettes ? Sur le canapé, peut-être ? Mila monte un genou. Le coussin est vide. Dans mes mains ? Elle ouvre les paumes. Rien. Elles sont perdues. Les cubes sont encore au pied. Je veux voir dessous. Mila prend un cube. Elle le pose dans la caisse. Toc. Une petite voiture attend aussi. Elle va dans la caisse. Toc.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le métal du radiateur fait psss. Une lampe ronde pose un halo. Mila connaît ce salon, le soir. Un détail paraît nouveau, sur le métal. Au campement du radiateur, ça sent le bois. Des chaussettes de laine attendent. Elles sont épaisses, près du canapé. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de laine&lt;/emphasis&gt; brille. Il est petit, papa. C'est un éclat de laine. La laine sent le linge propre. Les chaussettes sont chaudes, Mila. On les laisse près du chaud. Une caisse en bois est là. Elle sent un peu la forêt. Le tapis est froid, sous les orteils. J'ai froid aux pieds ! Je veux les chaussettes, maintenant ! Avant la tour de cubes ? Non, les chaussettes d'abord ! En ce moment, Mila saisit la laine. La laine est chaude, un peu lourde. Un cube rouge attend au sol. Une tour petite, aussi ! Elle pose un cube trop vite. Ça fait clic, contre le tapis. Puis un cube jaune. Ça fait clic, contre le rouge. Ta tour est jolie. Elle est petite, papa. Mila pose un cube de plus. La tour penche vers la laine. Deux cubes glissent. Ils tombent sur les chaussettes. Oh. Le sourire de Mila disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Où sont mes chaussettes ? Sur le canapé, peut-être ? Mila monte un genou. Le coussin est vide. Dans mes mains ? Elle ouvre les paumes. Rien. Elles sont perdues. Je prends tout, d'un coup ! Elle saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Constantin joue dans le salon. Les cubes sont partout. Papa dit : on range. Les jouets retournent dans la caisse. Constantin prend un cube. Il le met dans la caisse. Il prend une voiture. Il la met dans la caisse. Papa aide. Ils rangent ensemble. La caisse se remplit. Le tapis redevient vide. Constantin dit : j'ai rangé. Papa sourit. Constantin pousse la caisse. La caisse va près du meuble. &lt;emphasis&gt;ranger&lt;/emphasis&gt;, c'est mettre dans la caisse. Papa dit : merci. Constantin tape des mains.&lt;/slow&gt; [pause]</t>
+          <t>Le métal du radiateur fait psss. Une lampe ronde pose un halo. Mila connaît ce salon, le soir. Un détail paraît nouveau, sur le métal. Au campement du radiateur, ça sent le bois. Des chaussettes de laine attendent. Elles sont épaisses, près du canapé. Sur le bord, un &lt;emphasis&gt;éclat de laine&lt;/emphasis&gt; brille. Il est petit, papa. C'est un éclat de laine. La laine sent le linge propre. Les chaussettes sont chaudes, Mila. On les laisse près du chaud. Une caisse en bois est là. Elle sent un peu la forêt. Le tapis est froid, sous les orteils. J'ai froid aux pieds ! Je veux les chaussettes, maintenant ! Avant la tour de cubes ? Non, les chaussettes d'abord ! En ce moment, Mila saisit la laine. La laine est chaude, un peu lourde. Un cube rouge attend au sol. Une tour petite, aussi ! Elle pose un cube trop vite. Ça fait clic, contre le tapis. Puis un cube jaune. Ça fait clic, contre le rouge. Ta tour est jolie. Elle est petite, papa. Mila pose un cube de plus. La tour penche vers la laine. Deux cubes glissent. Ils tombent sur les chaussettes. Oh. Le sourire de Mila disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Où sont mes chaussettes ? Sur le canapé, peut-être ? Mila monte un genou. Le coussin est vide. Dans mes mains ? Elle ouvre les paumes. Rien. Elles sont perdues. Je prends tout, d'un coup ! Elle saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat de laine</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,46 +1319,52 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_chaussettes_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le radiateur chante un tout petit air.
-narrateur|Psss.
+          <t>narrateur|Le métal du radiateur fait psss.
+narrateur|Une lampe ronde pose un halo.
+narrateur|Mila connaît ce salon, le soir.
+narrateur|Un détail paraît nouveau, sur le métal.
+narrateur|Au campement du radiateur, ça sent le bois.
 narrateur|Des chaussettes de laine attendent.
 narrateur|Elles sont épaisses, près du canapé.
-narrateur|Elles sentent le linge propre.
-maman|Les chaussettes sont chaudes, papa.
-papa|Oui, on les laisse près du chaud.
-narrateur|Une caisse en bois est au salon.
+narrateur|Sur le bord, un éclat de laine brille.
+enfant-f|Il est petit, papa.
+papa|C'est un éclat de laine.
+narrateur|La laine sent le linge propre.
+maman|Les chaussettes sont chaudes, Mila.
+papa|On les laisse près du chaud.
+narrateur|Une caisse en bois est là.
 narrateur|Elle sent un peu la forêt.
-narrateur|En ce moment, Mila est près du canapé.
-narrateur|Elle touche un cube.
-narrateur|Le cube est lisse.
-enfant-f|Il est chaud, papa.
-papa|C'est le radiateur, Mila.
-enfant-f|Je fais une petite tour.
-maman|Une tour, avant les chaussettes ?
-enfant-f|Oui, une tour petite.
-narrateur|Mila pose un cube.
-narrateur|Puis un autre cube.
-narrateur|Clic.
-narrateur|Elle fait une petite tour.
+narrateur|Le tapis est froid, sous les orteils.
+enfant-f|J'ai froid aux pieds !
+enfant-f|Je veux les chaussettes, maintenant !
+maman|Avant la tour de cubes ?
+enfant-f|Non, les chaussettes d'abord !
+narrateur|En ce moment, Mila saisit la laine.
+narrateur|La laine est chaude, un peu lourde.
+narrateur|Un cube rouge attend au sol.
+enfant-f|Une tour petite, aussi !
+narrateur|Elle pose un cube trop vite.
+narrateur|Ça fait clic, contre le tapis.
+narrateur|Puis un cube jaune.
+narrateur|Ça fait clic, contre le rouge.
 papa|Ta tour est jolie.
 enfant-f|Elle est petite, papa.
-narrateur|Mila pose un cube rouge.
-narrateur|Clic.
-narrateur|La tour grandit un peu.
-narrateur|Ses pieds sont près du radiateur.
-enfant-f|Après, les chaussettes chaudes.
-maman|Oui, pour les orteils.
-narrateur|Mila pose encore un cube.
-narrateur|La tour penche vers les chaussettes.
+narrateur|Mila pose un cube de plus.
+narrateur|La tour penche vers la laine.
 narrateur|Deux cubes glissent.
-narrateur|Ils tombent sur la laine.
+narrateur|Ils tombent sur les chaussettes.
 enfant-f|Oh.
-papa|La tour a bougé.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, envie et inquiétude se bousculent.
 enfant-f|Où sont mes chaussettes ?
 maman|Sur le canapé, peut-être ?
 narrateur|Mila monte un genou.
@@ -1367,14 +1373,19 @@
 narrateur|Elle ouvre les paumes.
 narrateur|Rien.
 enfant-f|Elles sont perdues.
-papa|Les cubes sont encore au pied.
-enfant-f|Je veux voir dessous.
-narrateur|Mila prend un cube.
-narrateur|Elle le pose dans la caisse.
-narrateur|Toc.
-narrateur|Une petite voiture attend aussi.
-narrateur|Elle va dans la caisse.
-narrateur|Toc.</t>
+enfant-f|Je prends tout, d'un coup !
+narrateur|Elle saisit la pile trop vite.
+narrateur|Les cubes glissent entre ses doigts.
+narrateur|Le tapis disparaît sous les cubes.
+enfant-f|Ça ne veut pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes sous les cubes ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>radiateur,laine</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1417,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila cherche ses chaussettes. Où sont-elles ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila cherche ses &lt;emphasis level="moderate"&gt;chaussettes&lt;/emphasis&gt;. Où sont-elles ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le jeu est fini. Que fait Constantin ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila cherche ses &lt;emphasis&gt;chaussettes&lt;/emphasis&gt;. Où sont-elles ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1474,7 +1485,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,10 +1493,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1500,34 +1511,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>chaussettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,13 +1551,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1552,7 +1567,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_chaussettes_sont_sous_les_cubes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1585,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Un cube rouge reste au sol. Mila le glisse dans la caisse. Toc. Tu regardes bien sous la tour ? Oui, maman. Un bout de tapis reparaît. Encore un, tout doux. Mila écarte le dernier cube. Un coin de laine épaisse. Mes chaussettes ! Les chaussettes étaient sous la tour. Elles sont encore chaudes. Mila les serre contre sa joue. La laine sent le savon. Merci, tu les as trouvées. Te voilà, petite laine. Elles étaient dessous. La caisse a les cubes, maintenant. Le tapis près du radiateur est libre. Le radiateur chante encore un peu.</t>
+          <t>Mila refuse de prendre toute la pile. Elle pose un genou au tapis. Un cube rouge reste près de sa main. Je le mets toute seule. Elle glisse le cube dans la caisse. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Le cube jaune va dans la caisse. Toc. Je sors le reste, d'un coup ! Elle tire trop fort sur un cube. Deux cubes retombent, comme un toit. Oh. Mila ne reprend pas trop vite. Elle écoute le salon, un instant. Le radiateur fait psss, près d'elle. Sous un cube, un éclat de laine brille. Il est là. Mila refuse de foncer. Elle écarte un cube, lentement. Un coin de laine épaisse. Mes chaussettes ! Les chaussettes étaient sous la tour. Elles sentent le savon, un peu chaud. Mila les serre contre sa joue. Merci, Mila. Elles étaient dessous. La caisse a presque tous les cubes. Une petite voiture va dedans. Toc. Le tapis est libre, près du chaud. La laine peut s'enfiler ? Oui, maman. Mila pose la main sur la laine. Le tissu est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Un cube rouge reste au sol. Mila le glisse dans la caisse. Toc. Tu regardes bien sous la tour ? Oui, maman. Un bout de tapis reparaît. Encore un, tout doux. Mila écarte le dernier cube. Un coin de laine épaisse. Mes chaussettes ! Les chaussettes étaient sous la tour. Elles sont encore chaudes. Mila les serre contre sa joue. La laine sent le savon. Merci, tu les as trouvées. Te voilà, petite laine. Elles étaient dessous. La caisse a les cubes, maintenant. Le tapis près du radiateur est libre. Le radiateur chante encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila refuse de prendre toute la pile. Elle pose un genou au tapis. Un cube rouge reste près de sa main. Je le mets toute seule. Elle glisse le cube dans la &lt;emphasis level="moderate"&gt;caisse&lt;/emphasis&gt;. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Le cube jaune va dans la caisse. Toc. Je sors le reste, d'un coup ! Elle tire trop fort sur un cube. Deux cubes retombent, comme un toit. Oh. Mila ne reprend pas trop vite. Elle écoute le salon, un instant. Le radiateur fait psss, près d'elle. Sous un cube, un éclat de laine brille. Il est là. Mila refuse de foncer. Elle écarte un cube, lentement. Un coin de laine épaisse. Mes chaussettes ! Les chaussettes étaient sous la tour. Elles sentent le savon, un peu chaud. Mila les serre contre sa joue. Merci, Mila. Elles étaient dessous. La caisse a presque tous les cubes. Une petite voiture va dedans. Toc. Le tapis est libre, près du chaud. La laine peut s'enfiler ? Oui, maman. Mila pose la main sur la laine. Le tissu est un peu rêche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Constantin a rangé. Les cubes sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Papa a aidé.&lt;/slow&gt; [pause]</t>
+          <t>Mila refuse de prendre toute la pile. Elle pose un genou au tapis. Un cube rouge reste près de sa main. Je le mets toute seule. Elle glisse le cube dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Toc. Le bois sent un peu la forêt. Tu regardes bien dessous ? Oui, maman. La tour devient plus petite. Un bout de tapis reparaît. Le cube jaune va dans la caisse. Toc. Je sors le reste, d'un coup ! Elle tire trop fort sur un cube. Deux cubes retombent, comme un toit. Oh. Mila ne reprend pas trop vite. Elle écoute le salon, un instant. Le radiateur fait psss, près d'elle. Sous un cube, un éclat de laine brille. Il est là. Mila refuse de foncer. Elle écarte un cube, lentement. Un coin de laine épaisse. Mes chaussettes ! Les chaussettes étaient sous la tour. Elles sentent le savon, un peu chaud. Mila les serre contre sa joue. Merci, Mila. Elles étaient dessous. La caisse a presque tous les cubes. Une petite voiture va dedans. Toc. Le tapis est libre, près du chaud. La laine peut s'enfiler ? Oui, maman. Mila pose la main sur la laine. Le tissu est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,7 +1657,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1650,10 +1665,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1683,23 +1698,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1708,10 +1723,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,35 +1735,59 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_pose_un_cube_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Un cube rouge reste au sol.
-narrateur|Mila le glisse dans la caisse.
+          <t>narrateur|Mila refuse de prendre toute la pile.
+narrateur|Elle pose un genou au tapis.
+narrateur|Un cube rouge reste près de sa main.
+enfant-f|Je le mets toute seule.
+narrateur|Elle glisse le cube dans la caisse.
 narrateur|Toc.
-maman|Tu regardes bien sous la tour ?
+narrateur|Le bois sent un peu la forêt.
+maman|Tu regardes bien dessous ?
 enfant-f|Oui, maman.
+narrateur|La tour devient plus petite.
 narrateur|Un bout de tapis reparaît.
-papa|Encore un, tout doux.
-narrateur|Mila écarte le dernier cube.
+narrateur|Le cube jaune va dans la caisse.
+narrateur|Toc.
+enfant-f|Je sors le reste, d'un coup !
+narrateur|Elle tire trop fort sur un cube.
+narrateur|Deux cubes retombent, comme un toit.
+enfant-f|Oh.
+narrateur|Mila ne reprend pas trop vite.
+narrateur|Elle écoute le salon, un instant.
+narrateur|Le radiateur fait psss, près d'elle.
+narrateur|Sous un cube, un éclat de laine brille.
+enfant-f|Il est là.
+narrateur|Mila refuse de foncer.
+narrateur|Elle écarte un cube, lentement.
 narrateur|Un coin de laine épaisse.
 enfant-f|Mes chaussettes !
 narrateur|Les chaussettes étaient sous la tour.
-narrateur|Elles sont encore chaudes.
+narrateur|Elles sentent le savon, un peu chaud.
 narrateur|Mila les serre contre sa joue.
-narrateur|La laine sent le savon.
-papa|Merci, tu les as trouvées.
-maman|Te voilà, petite laine.
+papa|Merci, Mila.
 enfant-f|Elles étaient dessous.
-narrateur|La caisse a les cubes, maintenant.
-narrateur|Le tapis près du radiateur est libre.
-narrateur|Le radiateur chante encore un peu.</t>
+narrateur|La caisse a presque tous les cubes.
+narrateur|Une petite voiture va dedans.
+narrateur|Toc.
+narrateur|Le tapis est libre, près du chaud.
+maman|La laine peut s'enfiler ?
+enfant-f|Oui, maman.
+narrateur|Mila pose la main sur la laine.
+narrateur|Le tissu est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,bois</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1814,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman tend les chaussettes. Mila enfile la première. Puis la deuxième. Elles sont douces. Les orteils sont au chaud. Mila s'assoit près du radiateur. Le métal chante tout bas. On reste un moment ? Oui, maman. Ses pieds touchent le tapis libre. La laine est épaisse, un peu lourde. Tu veux le livre du canard ? Oui, papa. Papa ouvre le livre. La couverture est lisse. Mila pose un pied sur l'autre. Les chaussettes restent bien chaudes.</t>
+          <t>On enfile les chaussettes ? Maman tend la première. Mila pousse le pied, trop vite. La laine se plie, de travers. Elle ne veut pas ! Mila veut foncer, d'un coup. Mila refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde le bord de laine. Un éclat de laine brille, au revers. Comme sur le métal ! Tu le vois, toi ? Oui, sur ce bord. Mila tourne la chaussette, lente. Elle écoute le radiateur, un instant. Psss. Le pied glisse, sans forcer. Elle est dedans. Et l'autre ? La deuxième suit, sans se presser. Les orteils sont au chaud ? Oui, papa. Mila s'assoit près du radiateur. Le métal chante, petit. Tu veux le livre du canard ? Oui, papa. Papa ouvre le livre. La couverture est lisse. Les pieds touchent le tapis libre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman tend les chaussettes. Mila enfile la première. Puis la deuxième. Elles sont douces. Les orteils sont au chaud. Mila s'assoit près du radiateur. Le métal chante tout bas. On reste un moment ? Oui, maman. Ses pieds touchent le tapis libre. La laine est épaisse, un peu lourde. Tu veux le livre du canard ? Oui, papa. Papa ouvre le livre. La couverture est lisse. Mila pose un pied sur l'autre. Les chaussettes restent bien chaudes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;On enfile les chaussettes ? Maman tend la première. Mila pousse le pied, trop vite. La laine se plie, de travers. Elle ne veut pas ! Mila veut foncer, d'un coup. Mila refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde le bord de laine. Un &lt;emphasis level="moderate"&gt;éclat de laine&lt;/emphasis&gt; brille, au revers. Comme sur le métal ! Tu le vois, toi ? Oui, sur ce bord. Mila tourne la chaussette, lente. Elle écoute le radiateur, un instant. Psss. Le pied glisse, sans forcer. Elle est dedans. Et l'autre ? La deuxième suit, sans se presser. Les orteils sont au chaud ? Oui, papa. Mila s'assoit près du radiateur. Le métal chante, petit. Tu veux le livre du canard ? Oui, papa. Papa ouvre le livre. La couverture est lisse. Les pieds touchent le tapis libre.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Constantin s'assoit près de papa. Le salon est calme.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;On enfile les chaussettes ? Maman tend la première. Mila pousse le pied, trop vite. La laine se plie, de travers. Elle ne veut pas ! Mila veut foncer, d'un coup. Mila refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde le bord de laine. Un &lt;emphasis&gt;éclat de laine&lt;/emphasis&gt; brille, au revers. Comme sur le métal ! Tu le vois, toi ? Oui, sur ce bord. Mila tourne la chaussette, lente. Elle écoute le radiateur, un instant. Psss. Le pied glisse, sans forcer. Elle est dedans. Et l'autre ? La deuxième suit, sans se presser. Les orteils sont au chaud ? Oui, papa. Mila s'assoit près du radiateur. Le métal chante, petit. Tu veux le livre du canard ? Oui, papa. Papa ouvre le livre. La couverture est lisse. Les pieds touchent le tapis libre.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,7 +1871,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1840,22 +1879,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1864,28 +1907,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de laine</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1894,40 +1941,63 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman tend les chaussettes.
-narrateur|Mila enfile la première.
-narrateur|Puis la deuxième.
-enfant-f|Elles sont douces.
-papa|Les orteils sont au chaud.
+          <t>maman|On enfile les chaussettes ?
+narrateur|Maman tend la première.
+narrateur|Mila pousse le pied, trop vite.
+narrateur|La laine se plie, de travers.
+enfant-f|Elle ne veut pas !
+narrateur|Mila veut foncer, d'un coup.
+narrateur|Mila refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Elle regarde le bord de laine.
+narrateur|Un éclat de laine brille, au revers.
+enfant-f|Comme sur le métal !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur ce bord.
+narrateur|Mila tourne la chaussette, lente.
+narrateur|Elle écoute le radiateur, un instant.
+narrateur|Psss.
+narrateur|Le pied glisse, sans forcer.
+enfant-f|Elle est dedans.
+maman|Et l'autre ?
+narrateur|La deuxième suit, sans se presser.
+papa|Les orteils sont au chaud ?
+enfant-f|Oui, papa.
 narrateur|Mila s'assoit près du radiateur.
-narrateur|Le métal chante tout bas.
-maman|On reste un moment ?
-enfant-f|Oui, maman.
-narrateur|Ses pieds touchent le tapis libre.
-narrateur|La laine est épaisse, un peu lourde.
+narrateur|Le métal chante, petit.
 papa|Tu veux le livre du canard ?
 enfant-f|Oui, papa.
 narrateur|Papa ouvre le livre.
 narrateur|La couverture est lisse.
-narrateur|Mila pose un pied sur l'autre.
-narrateur|Les chaussettes restent bien chaudes.</t>
+narrateur|Les pieds touchent le tapis libre.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>chaussettes,livre</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2024,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mes pieds sont au chaud. La laine a été retrouvée. Bravo, tu les as trouvées. Le radiateur chante encore. La laine reste douce sur les orteils.</t>
+          <t>Ils restent près du campement du radiateur. La chaleur touche les orteils de Mila. Mes pieds sont au chaud. Oui, la laine est là. Un coin de laine porte une trace claire. Comme l'éclat de laine, papa ! Tu le vois, toi ? Oui, sur mon orteil. Mila glisse un pied sur l'autre. La laine repose, un peu lourde. On le sent, maman. Tu le sens sur tes orteils ? Oui, il est chaud. Le livre du canard reste ouvert. L'éclat de laine tient sur l'orteil.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mes pieds sont au chaud. La laine a été retrouvée. Bravo, tu les as trouvées. Le radiateur chante encore. La laine reste douce sur les orteils.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du campement du radiateur. La chaleur touche les orteils de Mila. Mes pieds sont au chaud. Oui, la laine est là. Un coin de laine porte une trace claire. Comme l'&lt;emphasis level="moderate"&gt;éclat de laine&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur mon orteil. Mila glisse un pied sur l'autre. La laine repose, un peu lourde. On le sent, maman. Tu le sens sur tes orteils ? Oui, il est chaud. Le livre du canard reste ouvert. L'éclat de laine tient sur l'orteil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du campement du radiateur. La chaleur touche les orteils de Mila. Mes pieds sont au chaud. Oui, la laine est là. Un coin de laine porte une trace claire. Comme l'&lt;emphasis&gt;éclat de laine&lt;/emphasis&gt;, papa ! Tu le vois, toi ? Oui, sur mon orteil. Mila glisse un pied sur l'autre. La laine repose, un peu lourde. On le sent, maman. Tu le sens sur tes orteils ? Oui, il est chaud. Le livre du canard reste ouvert. L'éclat de laine tient sur l'orteil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2081,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2101,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2115,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de laine</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2138,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,28 +2151,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_orteil; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Mes pieds sont au chaud.
-maman|La laine a été retrouvée.
-papa|Bravo, tu les as trouvées.
-narrateur|Le radiateur chante encore.
-narrateur|La laine reste douce sur les orteils.</t>
+          <t>narrateur|Ils restent près du campement du radiateur.
+narrateur|La chaleur touche les orteils de Mila.
+enfant-f|Mes pieds sont au chaud.
+maman|Oui, la laine est là.
+narrateur|Un coin de laine porte une trace claire.
+enfant-f|Comme l'éclat de laine, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur mon orteil.
+narrateur|Mila glisse un pied sur l'autre.
+narrateur|La laine repose, un peu lourde.
+enfant-f|On le sent, maman.
+maman|Tu le sens sur tes orteils ?
+enfant-f|Oui, il est chaud.
+narrateur|Le livre du canard reste ouvert.
+narrateur|L'éclat de laine tient sur l'orteil.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur,laine</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2211,6 +2304,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>